<commit_message>
Fall back to local BLAST+ and fix live-test gaps
When another remote RID would pass the 24-hour limit, remaining batches run on local NCBI BLAST+ instead of the web service. Ship the Excel task pane in the wheel, stop RID waits after a configurable limit, merge the weekend off-hours window, and do not count reused RIDs.

Co-authored-by: Topabaem <Topabaem05@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/blastid/data/default.xlsx
+++ b/src/blastid/data/default.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$U$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$V$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -464,8 +464,9 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="60" customWidth="1" min="19" max="19"/>
-    <col width="60" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="60" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -566,17 +567,22 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>검색 출처</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>검토 코멘트 / 스크린샷</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>스크린샷 (링크)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U1"/>
+  <autoFilter ref="A1:V1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>